<commit_message>
0.7.2-dev: APC props merged without E/EP suffix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/HangarLab template.xlsx
+++ b/tools/HangarLab template.xlsx
@@ -1563,7 +1563,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
@@ -1934,7 +1934,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>APC 16x8E</t>
+          <t>APC 16x8</t>
         </is>
       </c>
       <c r="B2" s="5" t="n">

</xml_diff>